<commit_message>
Add Batch 5 school scraping (CalArts, UCLA, Columbia College Chicago)
Final batch — all 28 schools from art_school_scraping_urls.md now
investigated. Master workbook reaches 22 tabs / 1,840 students. Cooper
Union and SCAD confirmed as dead ends/non-current data respectively and
were not scraped; Cornell and Alfred (from earlier batches) remain the
other unresolved sources.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -26,6 +26,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCA" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MassArt" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="U Michigan Stamps" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalArts" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UCLA" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columbia College Chicago" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$I$326</definedName>
@@ -47,6 +50,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CCA'!$A$5:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'U Michigan Stamps'!$A$5:$I$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'CalArts'!$A$5:$I$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'UCLA'!$A$5:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Columbia College Chicago'!$A$5:$I$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42546,6 +42552,3557 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: CalArts 'High Pass' BFA Class of 2026 group exhibition page (names only; site requires crawl4ai due to cookie-consent/Cloudflare Turnstile blocking a plain fetch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rita Aldridge</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Adrian Anguiano</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Elyse Beavers</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Raven Bridgewaters</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jessica Yuexi Chen</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Indie Courtney</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Xochitl Quetzalli Cruz</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sophie Darling</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ivan Nuñez DelaCruz</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Angharad Fitzgerald</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Jonathan Jin</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Amaris Jordan</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Riley Kate</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sadira Kuelling</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mackenzie Lord</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Eugenia Moreeva</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ethan Nahman</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mike Nott</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Elizaveta Novikova</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Okey Ofomata</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Natalee Park</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Suzy Park</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Abraham Perez</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ella Rose</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Solomon Rosenthal</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Frances Sheehy</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Elliot Smolin</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Marisa del toro</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>QQ Yi</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BFA Art / Photo Media</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>CalArts</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Name only, from 'High Pass' BFA Class of 2026 group exhibition page; no email/portfolio published on source page</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I34"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6:G34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: UCLA Department of Art — current Graduate Students directory by area of study (Ceramics, Interdisciplinary Studio, New Genres, Painting and Drawing, Photography, Sculpture), each linking to a personal portfolio/Instagram where available</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.art.ucla.edu/graduate-students</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dane Nakama</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.bydanenakama.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ethan Shaw</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/niceguysfinishinlast</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>g.aguilar magaña</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.geneaguilarstudio.com/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lynsey Robertson</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.lynseyjrobertson.com/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Utē Petit</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Victor Saucedo</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Felix Li</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MFA Interdisciplinary Studio</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lucas Wrench</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MFA Interdisciplinary Studio</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.lucaswrench.info</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sabaah Folayan</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MFA Interdisciplinary Studio</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://www.sabaah.is/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Vanessa Norton</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MFA Interdisciplinary Studio</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.vanessanorton.com/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>vincent hernandez</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MFA Interdisciplinary Studio</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Carlos Camacho</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MFA New Genres</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Emir West</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MFA New Genres</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Jazmin Jazzy Romero</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MFA New Genres</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.jazminromero.com/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Markele Cullins</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MFA New Genres</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://markelecullins.com/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Samar Al Summary</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MFA New Genres</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.samaralsummary.com</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Anja Salonen</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/anjasalonen/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Dilan Torres</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Gillian N Haigh</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://gilliannhaigh.com/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Jacqueline Valenzuela</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://jacquelinevalenzuela.com/</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jerry Alexis Peña</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/jerryalexispena</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Luke Francis Austin</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/l.f.austin/</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Magnus Maxine Flowers</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Roshini Agarwal</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/roshini_agarwal</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Tammy Chang</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://www.tammy-chang.com/</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Victor Ballesteros</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>http://instagram.com/vmballesterosg</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wihro Kim</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>No portfolio/social link listed for this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Alina van Ryzin</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alinavanryzin</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Andrés de Varona</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.andresmario.com/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Anne Vetter</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://www.acvetter.com/</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Ashley Michelle Hannah</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://ashleymichellehannah.com/</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Keegan Isaac Holden</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://www.keeganholden.com/</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>abhishek kulkarni</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MFA Sculpture</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/a.ar.kay/</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Andrew Sungtaek</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MFA Sculpture</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/a.sungtaek</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Aryana Polat</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MFA Sculpture</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://aryanapolat.com/</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>libbi ponce</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MFA Sculpture</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://libbiponce.com/</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>tunmi da silva</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MFA Sculpture</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://www.tunmidasilva.com/</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Yao Wang</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MFA Sculpture</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://wangyao.info/</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I43"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Columbia College Chicago — 'Human Condition' 2026 BA/BFA Fine Art Exhibition page, Hokin Gallery and C33 Gallery exhibitor lists (names only). Note: 2 of 24 names have unusual letter-spacing in the source HTML itself (e.g. 'Faith H o g a n') — kept verbatim, flagged in notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Jupiter Brodie</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Carley Brown</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fiona Connors</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jocelyn Diaz</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Faith H o g a n</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published; NOTE: name appears to have unusual letter-spacing in the source HTML itself (e.g. single letters separated by spaces) — kept verbatim, may not reflect the person's actual name spelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Emelia Kay</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Aja "Morningstar" Martin</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hai Martinez</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Frida Mejia</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Nat Slavin</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Brianna Wilkins</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Isa Woodard</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Liz Z e r m e n o Robles</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (Hokin Gallery)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Name only, from 'Hokin Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published; NOTE: name appears to have unusual letter-spacing in the source HTML itself (e.g. single letters separated by spaces) — kept verbatim, may not reflect the person's actual name spelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Jala Bowers</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Jenna Davis</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Trevell Hampton</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Alivia King</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ana Lara</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Drew Malapanes</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Elise N e a l</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published; NOTE: name appears to have unusual letter-spacing in the source HTML itself (e.g. single letters separated by spaces) — kept verbatim, may not reflect the person's actual name spelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wang Jing Yi (Eliana Pinkert)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cristian Romero</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Liza Smith</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Stefanie Valle Aguilera</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BFA/BA Fine Art (C33 Gallery)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Columbia College Chicago</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I29"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Batch 6 school scraping (Iowa, UW Art, BGSU) from new 31-70 doc
First batch from a new research doc listing 28 more schools (ranks
~31-70). Scoped to the doc's own "Tier 1" (cleanest, no-JS) picks per
user decision. UT Knoxville confirmed unreachable this session (AWS WAF
CAPTCHA on TRACE + connection timeouts across all fallback URLs).
Master workbook reaches 25 tabs / 1,874 students.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -29,6 +29,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalArts" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UCLA" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columbia College Chicago" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iowa" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UW Art" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BGSU" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$I$326</definedName>
@@ -53,6 +56,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'CalArts'!$A$5:$I$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'UCLA'!$A$5:$I$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Columbia College Chicago'!$A$5:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Iowa'!$A$5:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'UW Art'!$A$5:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$I$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46103,6 +46109,1638 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: University of Iowa School of Art, Art History, and Design — MFA Virtual Exhibitions page (2024-2026 cohorts), each linking to a Matterport 3D exhibition tour rather than a personal portfolio site</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://art.uiowa.edu/events/mfa-virtual-exhibitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Heather Steckler</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=bUQuRPrPXn5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cara Krippner</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=QMBBNq3N6VX</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Anna Roemerman</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA 3D Design</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=1RzXZaJURgK</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Antonia Baafi</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Jewelry and Metal Arts</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=E4APuduuJ7R</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lya Finston</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=PkmkecLPwnV</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Amanda Shepard</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Jewelry and Metal Arts</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=uCPoUCvVax8</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ben Eastman</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MFA 3D Design</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=1ncCV6yM24a</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Javier Espinosa Momox</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=gAnFZ1qj4mX</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Patrick Ryan</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=e6BTTHxyJVm</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Al-Qawi Nanavati</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=ZLZKMucHd3u</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gracie Baer</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MFA Sculpture &amp; Intermedia</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=59w5kkDgyys</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Braden Dexter</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MFA Graphic Design</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=c5LN5QkVjdo</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Agnes Harry Mills</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MFA Jewlery and Metal Arts</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=vccXRs9sB2o</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Kyle Agnew</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=3veaLSxJd3y</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sofia Echeverri</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=L2tVk5UcqYH</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Na'ah Gordon</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=8mfrTxRfsF9</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Jordan Ramsey Ismaiel</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MFA Painting and Drawing</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=Gt8PNGatZUC</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lauren Krukowski</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://my.matterport.com/show/?m=MbXETFgfm4h</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Portfolio URL is a Matterport 3D virtual exhibition tour, not a personal site; no email published on source page</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I23"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6:G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: University of Washington 2026 MFA + MDes Thesis Exhibition page (Henry Art Gallery) — names only; source does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Stephanie Alacon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Dahae Cheon</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Li-Yuan Chiou</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jeff Jiang</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Victoria Mackender</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Alex Moni-Sauri</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Oscar Pearson</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Chave Pichardo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Andrew Roibal</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ryan Walters</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I15"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6:G15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: BGSU ScholarWorks — School of Art MA and MFA Graduate Exhibitions, Portfolios, and Theses repository, 2025 cohort (thesis title + author name; portfolio_url is the repository record, not a personal site)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://scholarworks.bgsu.edu/ms_art/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Syed Fatmi</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://scholarworks.bgsu.edu/ms_art/542</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Thesis title: "OMNISYS"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nick Felaris</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://scholarworks.bgsu.edu/ms_art/543</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Thesis title: "Nick Felaris Master of Fine Arts"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Precious Gyekye</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://scholarworks.bgsu.edu/ms_art/544</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Thesis title: "Unraveling Silence"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Peter Kiladejo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://scholarworks.bgsu.edu/ms_art/545</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Thesis title: "Adetope Peter Kiladejo Master of Fine Arts"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rachel Krieger</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://scholarworks.bgsu.edu/ms_art/546</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Thesis title: "Rachel Krieger"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kamrun Mim</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://scholarworks.bgsu.edu/ms_art/547</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Thesis title: "Kamrun Mim"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I11"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6:G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6:H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add discovered email for BGSU student (Syed Fatmi)
First school in the email-discovery enrichment pass: searched for emails for
all 6 name-only BGSU students. Found 1 high-confidence match (Syed Fatmi, via
his own portfolio site), flagged 1 blocked lead for manual follow-up (Kamrun
Mim), and left 4 as genuine no-finds rather than guessing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -47499,7 +47499,11 @@
           <t>Syed Fatmi</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>syedway.digital@gmail.com</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MFA Studio Art</t>
@@ -47512,7 +47516,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://scholarworks.bgsu.edu/ms_art/542</t>
+          <t>https://syedway.com/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -47528,7 +47532,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Thesis title: "OMNISYS"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+          <t>Thesis title: "OMNISYS"; email and portfolio found via web search (personal site syedway.com, confirmed via matching thesis title/LinkedIn)</t>
         </is>
       </c>
     </row>
@@ -47707,7 +47711,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://scholarworks.bgsu.edu/ms_art/547</t>
+          <t>https://kamrunnahermim.com/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -47723,7 +47727,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Thesis title: "Kamrun Mim"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+          <t>Thesis title: "Kamrun Mim"; personal site found via web search (kamrunnahermim.com) but returned HTTP 403 on fetch — could not retrieve email; try visiting contact page manually</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 3 more user-confirmed BGSU emails (Nick Felaris, Rachel Krieger, Kamrun Mim)
BGSU email discovery now at 4/6: user manually resolved 3 ambiguous/blocked
cases that automated search alone couldn't confirm.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -47542,7 +47542,11 @@
           <t>Nick Felaris</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nickfelaris@hotmail.com</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MFA Studio Art</t>
@@ -47571,7 +47575,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Thesis title: "Nick Felaris Master of Fine Arts"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+          <t>Thesis title: "Nick Felaris Master of Fine Arts"; email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -47659,7 +47663,11 @@
           <t>Rachel Krieger</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>rachelle@rachellekrieger.com</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MFA Studio Art</t>
@@ -47672,7 +47680,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://scholarworks.bgsu.edu/ms_art/546</t>
+          <t>https://www.rachellekrieger.com/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -47688,7 +47696,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Thesis title: "Rachel Krieger"; no email/personal portfolio published on source page (portfolio_url is the ScholarWorks repository record)</t>
+          <t>Thesis title: "Rachel Krieger"; email and portfolio confirmed by user via rachellekrieger.com contact page</t>
         </is>
       </c>
     </row>
@@ -47698,7 +47706,11 @@
           <t>Kamrun Mim</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>kamrunmim.print@gmail.com</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MFA Studio Art</t>
@@ -47711,7 +47723,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://kamrunnahermim.com/</t>
+          <t>https://kamrunnahermim.wordpress.com/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -47727,7 +47739,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Thesis title: "Kamrun Mim"; personal site found via web search (kamrunnahermim.com) but returned HTTP 403 on fetch — could not retrieve email; try visiting contact page manually</t>
+          <t>Thesis title: "Kamrun Mim"; email and portfolio confirmed by user via kamrunnahermim.wordpress.com/about (bio/CV section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email discovery pass for UW Art: no confirmed emails, 2 manual-check leads flagged
Searched all 10 UW Art (Henry Art Gallery) students. No email could be
confirmed automatically. Found personal sites for Victoria Mackender
(vamack.com) and Ryan Walters (ryanwalters.art) but this session's fetch tool
can't resolve those domains (DNS failure) -- flagged in notes for manual
follow-up. Other leads (Jeff Jiang, Oscar Pearson) have sites but no visible
email in static HTML.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -47137,7 +47137,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+          <t>https://jeff-jiang.com/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -47153,7 +47153,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+          <t>Personal site found via web search (jeff-jiang.com, footwear/product design background) but no email visible in static HTML — likely a JS-rendered contact form; no email found</t>
         </is>
       </c>
     </row>
@@ -47176,7 +47176,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+          <t>https://www.vamack.com/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -47192,7 +47192,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+          <t>Personal site found via web search (vamack.com) but this tool's fetcher could not resolve the domain (DNS failure) — try visiting manually for contact info; also has Instagram @vamackender</t>
         </is>
       </c>
     </row>
@@ -47254,7 +47254,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+          <t>https://oscarpearsonart.wixsite.com/studio</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -47270,7 +47270,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+          <t>Personal site found via web search (Wix site, Instagram @oscarpearson_) but no email visible — only a Wix contact form; no email found. NOTE: a different, unrelated Oscar Pearson (California muralist/gallery artist) also shows up in search — not to be confused with this student</t>
         </is>
       </c>
     </row>
@@ -47371,7 +47371,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+          <t>https://www.ryanwalters.art/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -47387,7 +47387,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+          <t>Personal site found via web search (ryanwalters.art) but this tool's fetcher could not resolve the .art domain (DNS failure) — try visiting manually for contact info</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add discovered emails for 4 MassArt students
Found high-confidence emails for Olivia Greenberg, Anastasia Sierra,
Shailee Thakkar, and Antonio Bailey via their own portfolio sites. Flagged
one unverified lead (Suzi Grossman) and left 6 as genuine no-finds.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -31338,7 +31338,11 @@
           <t>Olivia Greenberg</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>oliviadylan129@gmail.com</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MFA Photography</t>
@@ -31351,7 +31355,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://calendar.massart.edu/event/2026-mfa-thesis-exhibition-PARTI</t>
+          <t>https://www.oliviadylanphotography.com/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -31367,7 +31371,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Name only, from 'FEATURED ARTISTS' list; no email/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site oliviadylanphotography.com contact page)</t>
         </is>
       </c>
     </row>
@@ -31377,7 +31381,11 @@
           <t>Anastasia Sierra</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>info@anastasiasierra.com</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MFA Photography</t>
@@ -31390,7 +31398,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://calendar.massart.edu/event/2026-mfa-thesis-exhibition-PARTI</t>
+          <t>https://www.anastasiasierra.com/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -31406,7 +31414,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Name only, from 'FEATURED ARTISTS' list; no email/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site anastasiasierra.com/about)</t>
         </is>
       </c>
     </row>
@@ -31429,7 +31437,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://calendar.massart.edu/event/2026-mfa-thesis-exhibition-PARTI</t>
+          <t>https://visura.co/lspencer/about</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -31445,7 +31453,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Name only, from 'FEATURED ARTISTS' list; no email/portfolio published on source page</t>
+          <t>Photographer/writer based in Winchester, MA; Visura profile found via web search but returned HTTP 403 on fetch — no email found</t>
         </is>
       </c>
     </row>
@@ -31455,7 +31463,11 @@
           <t>Shailee Thakkar</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>shailee.v.thakkar@gmail.com</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MFA Studio Arts</t>
@@ -31468,7 +31480,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://calendar.massart.edu/event/2026-mfa-thesis-exhibition-PARTI</t>
+          <t>https://www.shaileethakkar.com/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -31484,7 +31496,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Name only, from 'FEATURED ARTISTS' list; no email/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site shaileethakkar.com/aboutme footer)</t>
         </is>
       </c>
     </row>
@@ -31533,7 +31545,11 @@
           <t>Antonio Bailey</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>antoniobaileylocal@gmail.com</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MFA Photography</t>
@@ -31546,7 +31562,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://calendar.massart.edu/event/2026-spring-mfa-thesis-exhibition-part-ii</t>
+          <t>https://www.antoniobailey.com/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -31562,7 +31578,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Name only, from 'FEATURED ARTISTS' list; no email/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site antoniobailey.com/about)</t>
         </is>
       </c>
     </row>
@@ -31585,7 +31601,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://calendar.massart.edu/event/2026-spring-mfa-thesis-exhibition-part-ii</t>
+          <t>https://camrynconnolly.com/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -31601,7 +31617,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Name only, from 'FEATURED ARTISTS' list; no email/portfolio published on source page</t>
+          <t>Personal site found via web search (camrynconnolly.com) but only a contact form is shown, no visible email; Instagram @camrynscollections</t>
         </is>
       </c>
     </row>
@@ -31624,7 +31640,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://calendar.massart.edu/event/2026-spring-mfa-thesis-exhibition-part-ii</t>
+          <t>https://www.suzigrossman.com/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -31640,7 +31656,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Name only, from 'FEATURED ARTISTS' list; no email/portfolio published on source page</t>
+          <t>UNVERIFIED possible email: Suzi@suzigrossman.com — surfaced via web search summary of the site's contact page, but the email is JS-obfuscated on the live page and could not be independently confirmed by direct fetch; not written as confirmed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add discovered emails for 3 CMU students (Al-Sarraj, Zito, Ford)
CMU now 11/14 with email. All 3 found via their own portfolio sites
(portfolio_url was already on file from the original scrape). Flagged 2
more leads (Yiying Wang, Walter Smits) whose sites exist but couldn't be
reached this session (DNS failure / site down).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -13205,7 +13205,11 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No email found — Behance profile has no listed contact info, no personal site found</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13271,7 +13275,11 @@
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Own site returned HTTP 503 (site appears down) on repeated fetch attempts; CMU directory page has no direct email listed — try visiting waltersmits.com manually</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13337,7 +13345,11 @@
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Own site (yiyingwang666.com) could not be resolved by this tool's fetcher (DNS failure) — try visiting manually; CMU directory page has no direct email listed</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13380,7 +13392,11 @@
           <t>Amber N. Ford</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>studio@ambernford.com</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MFA Studio Art (First-Year MFA)</t>
@@ -13389,7 +13405,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://art.cmu.edu/people/amber-ford/</t>
+          <t>https://www.ambernford.com/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -13403,7 +13419,11 @@
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site ambernford.com/info)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13446,7 +13466,11 @@
           <t>Sarah Al-Sarraj</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>info.sarahalsarraj@gmail.com</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MFA Studio Art (First-Year MFA)</t>
@@ -13469,7 +13493,11 @@
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site sarahalsarraj.com)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13617,7 +13645,11 @@
           <t>Stefanie Zito</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>info@stefaniezito.com</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MFA Studio Art (First-Year MFA)</t>
@@ -13640,7 +13672,11 @@
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site stefaniezito.com, listed as 'info[at]stefaniezito.com' anti-scrape format)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:I19"/>

</xml_diff>

<commit_message>
Add discovered emails for 5 Temple/Tyler students
Found high-confidence emails for Charles Jarboe, Amanda Crain-Freeland,
Rae Helms, Francesca Lally, and Lilly Buttitta via their own portfolio
sites (mostly on secondary bio/CV pages, not homepages). Flagged 4 more
real sites that couldn't be reached this session (403/DNS/503 failures)
for manual follow-up. Remaining ~21 students had no personal site or
contact info surfaced in search.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -68071,10 +68071,14 @@
           <t>Charles Jarboe</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>charles.jarboe@gmail.com</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Glass</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -68082,7 +68086,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.charles-jarboe.com/</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68096,7 +68104,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: February 26 - March 1); no email/major/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site charles-jarboe.com/bio)</t>
         </is>
       </c>
     </row>
@@ -68109,7 +68117,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Photography</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -68131,7 +68139,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: February 26 - March 1); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68166,7 +68174,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: February 26 - March 1); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68176,10 +68184,14 @@
           <t>Amanda Crain-Freeland</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>amandancrain@gmail.com</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Sculpture</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -68187,7 +68199,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.amandacrainfreeland.com/</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68201,7 +68217,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 12-March 15); no email/major/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site amandacrainfreeland.com CV page)</t>
         </is>
       </c>
     </row>
@@ -68214,7 +68230,7 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Sculpture</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -68222,7 +68238,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://fernandanunez.com/</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68236,7 +68256,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 12-March 15); no email/major/portfolio published on source page</t>
+          <t>Own site (fernandanunez.com) found via web search but returned HTTP 503 on fetch — try visiting manually</t>
         </is>
       </c>
     </row>
@@ -68249,7 +68269,7 @@
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Fiber/Sculpture</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -68257,7 +68277,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.mikaobayashi.com/</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68271,7 +68295,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 12-March 15); no email/major/portfolio published on source page</t>
+          <t>Personal site found via web search (mikaobayashi.com) but no email visible — only Instagram and a /contact link; no email found</t>
         </is>
       </c>
     </row>
@@ -68284,7 +68308,7 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -68306,7 +68330,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 12-March 15); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68319,7 +68343,7 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Photography</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -68327,7 +68351,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://sophiadellarciprete.com/</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68341,7 +68369,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 19 - March 22); no email/major/portfolio published on source page</t>
+          <t>Personal site found via web search (sophiadellarciprete.com) but no email visible in static HTML; no email found</t>
         </is>
       </c>
     </row>
@@ -68351,10 +68379,14 @@
           <t>Rae Helms</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Raehelmsprint@gmail.com</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Printmaking</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -68362,7 +68394,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://raehelms.ink/</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68376,7 +68412,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 19 - March 22); no email/major/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site raehelms.ink)</t>
         </is>
       </c>
     </row>
@@ -68386,10 +68422,14 @@
           <t>Francesca Lally</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>francescalally@gmail.com</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Printmaking</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -68397,7 +68437,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.francescalally.net/</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68411,7 +68455,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 19 - March 22); no email/major/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site francescalally.net/ccvv)</t>
         </is>
       </c>
     </row>
@@ -68424,7 +68468,7 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Ceramics</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -68432,7 +68476,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://arizuaro.com/</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68446,7 +68494,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 19 - March 22); no email/major/portfolio published on source page</t>
+          <t>Personal site found via web search (arizuaro.com) but no email visible — only Instagram link; no email found</t>
         </is>
       </c>
     </row>
@@ -68456,10 +68504,14 @@
           <t>Lilly Buttitta</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>lbuttittaart@gmail.com</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -68467,7 +68519,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://lillybuttitta.com/</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68481,7 +68537,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 26- March 29); no email/major/portfolio published on source page</t>
+          <t>Email and portfolio found via web search (own site lillybuttitta.com)</t>
         </is>
       </c>
     </row>
@@ -68494,7 +68550,7 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -68516,7 +68572,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 26- March 29); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced, only a LinkedIn profile</t>
         </is>
       </c>
     </row>
@@ -68551,7 +68607,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 26- March 29); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68586,7 +68642,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: March 26- March 29); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68621,7 +68677,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 2 - April 5); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68634,7 +68690,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Fiber and Material Studies</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -68642,7 +68698,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://maedehmehdipour.com/</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68656,7 +68716,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 2 - April 5); no email/major/portfolio published on source page</t>
+          <t>Personal site found via web search (maedehmehdipour.com) but returned HTTP 403 on fetch — could not retrieve email; try visiting manually</t>
         </is>
       </c>
     </row>
@@ -68669,7 +68729,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Printmaking</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -68691,7 +68751,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 2 - April 5); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — only a LinkedIn profile surfaced, no personal site</t>
         </is>
       </c>
     </row>
@@ -68726,7 +68786,7 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 2 - April 5); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68761,7 +68821,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 9 - April 12); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68796,7 +68856,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 9 - April 12); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68831,7 +68891,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 9 - April 12); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -68852,7 +68912,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.bensoloart.com/</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68866,7 +68930,7 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 9 - April 12); no email/major/portfolio published on source page</t>
+          <t>Own site (bensoloart.com) found via web search but could not be resolved by this tool's fetcher (DNS failure) — try visiting manually</t>
         </is>
       </c>
     </row>
@@ -68887,7 +68951,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://scoby.page/log3y-logan-crompton</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68901,7 +68969,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 16- April 19); no email/major/portfolio published on source page</t>
+          <t>Link-in-bio page (scoby.page) found via web search — not fetched for email this pass</t>
         </is>
       </c>
     </row>
@@ -68936,7 +69004,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 16- April 19); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced (full name may be 'Boi Boy Cottrell' per one source)</t>
         </is>
       </c>
     </row>
@@ -68949,7 +69017,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -68957,7 +69025,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://www.diegojuarez.com/</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68971,7 +69043,7 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 16- April 19); no email/major/portfolio published on source page</t>
+          <t>Personal site found via web search (diegojuarez.com/bio) but no email visible — only Instagram link and a /contact link not checked; no email found</t>
         </is>
       </c>
     </row>
@@ -68984,7 +69056,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -69006,7 +69078,7 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 16- April 19); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -69019,7 +69091,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Graphic Design</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -69041,7 +69113,7 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 23 - April 26); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced</t>
         </is>
       </c>
     </row>
@@ -69054,7 +69126,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Graphic Design</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -69076,7 +69148,7 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 23 - April 26); no email/major/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced; works at Running Press Book Publishers</t>
         </is>
       </c>
     </row>
@@ -69089,7 +69161,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Design</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -69097,7 +69169,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://pegahsaebi.com/</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -69111,7 +69187,7 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Name only, from exhibition schedule text (week: April 23 - April 26); no email/major/portfolio published on source page</t>
+          <t>Own site (pegahsaebi.com) found via web search but could not be resolved by this tool's fetcher (DNS failure) — try visiting manually</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 24 user-confirmed emails across UW Art, MassArt, CMU, and Temple/Tyler
User manually checked leads this session's tools couldn't reach (DNS
failures, 403/503 errors) plus several names with no automated lead at
all. Updated totals: UW Art 6/10, MassArt 6/11, CMU 13/14, Temple/Tyler
23/30. Confirms several tool-side DNS/fetch limitations were false
negatives, not dead sites.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -13252,7 +13252,11 @@
           <t>Walter Smits</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>smits.walt@gmail.com</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MFA Studio Art (First-Year MFA)</t>
@@ -13277,7 +13281,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Own site returned HTTP 503 (site appears down) on repeated fetch attempts; CMU directory page has no direct email listed — try visiting waltersmits.com manually</t>
+          <t>Email confirmed by user (site was returning HTTP 503 on repeated fetch attempts by this tool)</t>
         </is>
       </c>
     </row>
@@ -13322,7 +13326,11 @@
           <t>Yiying Wang</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>yiyingwang194@gmail.com</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MFA Studio Art (First-Year MFA)</t>
@@ -13347,7 +13355,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Own site (yiyingwang666.com) could not be resolved by this tool's fetcher (DNS failure) — try visiting manually; CMU directory page has no direct email listed</t>
+          <t>Email confirmed by user (site was unresolvable by this tool's fetcher)</t>
         </is>
       </c>
     </row>
@@ -31460,7 +31468,11 @@
           <t>Lisa Spencer</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>lisaspencergallery@gmail.com</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MFA Photography</t>
@@ -31489,7 +31501,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Photographer/writer based in Winchester, MA; Visura profile found via web search but returned HTTP 403 on fetch — no email found</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -31663,7 +31675,11 @@
           <t>Suzi Grossman</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Photo@suzigrossman.com</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MFA Photography</t>
@@ -31692,7 +31708,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>UNVERIFIED possible email: Suzi@suzigrossman.com — surfaced via web search summary of the site's contact page, but the email is JS-obfuscated on the live page and could not be independently confirmed by direct fetch; not written as confirmed</t>
+          <t>Email confirmed by user (different address than the earlier unverified search-summary guess)</t>
         </is>
       </c>
     </row>
@@ -47137,7 +47153,11 @@
           <t>Li-Yuan Chiou</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>lychiou@uw.edu</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MFA/MDes (UW Art — discipline not specified per student)</t>
@@ -47166,7 +47186,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+          <t>Email confirmed by user (UW address)</t>
         </is>
       </c>
     </row>
@@ -47215,7 +47235,11 @@
           <t>Victoria Mackender</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>victoriaa961@gmail.com</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MFA/MDes (UW Art — discipline not specified per student)</t>
@@ -47244,7 +47268,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Personal site found via web search (vamack.com) but this tool's fetcher could not resolve the domain (DNS failure) — try visiting manually for contact info; also has Instagram @vamackender</t>
+          <t>Email confirmed by user via vamack.com (manual check, DNS-unreachable by this tool)</t>
         </is>
       </c>
     </row>
@@ -47293,7 +47317,11 @@
           <t>Oscar Pearson</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>o2thescar@hotmail.com</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MFA/MDes (UW Art — discipline not specified per student)</t>
@@ -47322,7 +47350,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Personal site found via web search (Wix site, Instagram @oscarpearson_) but no email visible — only a Wix contact form; no email found. NOTE: a different, unrelated Oscar Pearson (California muralist/gallery artist) also shows up in search — not to be confused with this student</t>
+          <t>Email confirmed by user. NOTE: a different, unrelated Oscar Pearson (California muralist/gallery artist) also shows up in search — not to be confused with this student</t>
         </is>
       </c>
     </row>
@@ -47332,7 +47360,11 @@
           <t>Chave Pichardo</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>chavepichardostudios@gmail.com</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MFA/MDes (UW Art — discipline not specified per student)</t>
@@ -47361,7 +47393,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -47371,7 +47403,11 @@
           <t>Andrew Roibal</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AndrewRoibalArt@gmail.com</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MFA/MDes (UW Art — discipline not specified per student)</t>
@@ -47384,7 +47420,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+          <t>https://art.washington.edu/people/andrew-roibal</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -47400,7 +47436,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Name only, from Henry Art Gallery thesis exhibition page; no email/portfolio published; source page does not map a specific discipline to each individual student</t>
+          <t>Email confirmed by user (also has UW address aroibal@uw.edu)</t>
         </is>
       </c>
     </row>
@@ -47410,7 +47446,11 @@
           <t>Ryan Walters</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RyanWaltersFilms@gmail.com</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MFA/MDes (UW Art — discipline not specified per student)</t>
@@ -47439,7 +47479,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Personal site found via web search (ryanwalters.art) but this tool's fetcher could not resolve the .art domain (DNS failure) — try visiting manually for contact info</t>
+          <t>Email confirmed by user via ryanwalters.art (manual check, .art domain unreachable by this tool)</t>
         </is>
       </c>
     </row>
@@ -68114,7 +68154,11 @@
           <t>Natalia Purchiaroni</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>npurchphotography@gmail.com</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MFA Photography</t>
@@ -68139,7 +68183,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68149,7 +68193,11 @@
           <t>Macy West</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>macywest99@gmail.com</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68174,7 +68222,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68256,7 +68304,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Own site (fernandanunez.com) found via web search but returned HTTP 503 on fetch — try visiting manually</t>
+          <t>Own site (fernandanunez.com) found via web search but returned HTTP 503 on fetch; not resolved this pass — still needs manual check</t>
         </is>
       </c>
     </row>
@@ -68266,7 +68314,11 @@
           <t>Mika Obayashi</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>mikacobayashi@gmail.com</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MFA Fiber/Sculpture</t>
@@ -68295,7 +68347,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Personal site found via web search (mikaobayashi.com) but no email visible — only Instagram and a /contact link; no email found</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68305,7 +68357,11 @@
           <t>Heather Swenson</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mail@heatherswenson.com</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MFA Painting</t>
@@ -68316,7 +68372,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.heatherswenson.com/</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -68330,7 +68390,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user (own site heatherswenson.com)</t>
         </is>
       </c>
     </row>
@@ -68340,7 +68400,11 @@
           <t>Sophia Dell'Arciprete</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>sophiadellarciprete@yahoo.com</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MFA Photography</t>
@@ -68369,7 +68433,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Personal site found via web search (sophiadellarciprete.com) but no email visible in static HTML; no email found</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68465,7 +68529,11 @@
           <t>Ari Zuaro</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>azuaro@theclaystudio.org</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MFA Ceramics</t>
@@ -68494,7 +68562,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Personal site found via web search (arizuaro.com) but no email visible — only Instagram link; no email found</t>
+          <t>Email confirmed by user (Clay Studio staff address, where they also work)</t>
         </is>
       </c>
     </row>
@@ -68617,7 +68685,11 @@
           <t>Esther Park</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>eyparkart7@gmail.com</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68642,7 +68714,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68652,7 +68724,11 @@
           <t>Mollie Hansen</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>mollie.hansen.art@gmail.com</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68677,7 +68753,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68687,7 +68763,11 @@
           <t>Maedeh Mehdipour</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>mehdipour.maede@gmail.com</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MFA Fiber and Material Studies</t>
@@ -68716,7 +68796,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Personal site found via web search (maedehmehdipour.com) but returned HTTP 403 on fetch — could not retrieve email; try visiting manually</t>
+          <t>Email confirmed by user (site was returning HTTP 403 on fetch by this tool)</t>
         </is>
       </c>
     </row>
@@ -68761,7 +68841,11 @@
           <t>Madeline Rodriguez</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>rodriguez.maddie@gmail.com</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68786,7 +68870,7 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68831,7 +68915,11 @@
           <t>Ivy Jewell</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ijewell@theclaystudio.org</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68856,7 +68944,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user (Clay Studio staff address)</t>
         </is>
       </c>
     </row>
@@ -68866,7 +68954,11 @@
           <t>Angelique Scott</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ArtByAngeliqueScott@gmail.com</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68891,7 +68983,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -68901,7 +68993,11 @@
           <t>Ben Solo</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>benweidlich.bs@gmail.com</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68930,7 +69026,7 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Own site (bensoloart.com) found via web search but could not be resolved by this tool's fetcher (DNS failure) — try visiting manually</t>
+          <t>Email confirmed by user (real name appears to be Ben Weidlich; site was unresolvable by this tool's fetcher)</t>
         </is>
       </c>
     </row>
@@ -68940,7 +69036,11 @@
           <t>Logan Crompton</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>lcrompton@kcai.edu</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -68969,7 +69069,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Link-in-bio page (scoby.page) found via web search — not fetched for email this pass</t>
+          <t>Email confirmed by user (Kansas City Art Institute address)</t>
         </is>
       </c>
     </row>
@@ -68979,7 +69079,11 @@
           <t>Boi Boy</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>boiboy.art@gmail.com</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -69004,7 +69108,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced (full name may be 'Boi Boy Cottrell' per one source)</t>
+          <t>Email confirmed by user (full name may be 'Boi Boy Cottrell' per one source)</t>
         </is>
       </c>
     </row>
@@ -69014,7 +69118,11 @@
           <t>Diego Juarez</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>juarezcdiego@gmail.com</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>MFA Painting</t>
@@ -69043,7 +69151,7 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Personal site found via web search (diegojuarez.com/bio) but no email visible — only Instagram link and a /contact link not checked; no email found</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -69053,7 +69161,11 @@
           <t>Gianna Santucci</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>gsantucci630@gmail.com</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
           <t>MFA Painting</t>
@@ -69078,7 +69190,7 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>No email found via web search — no personal site surfaced</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
@@ -69158,7 +69270,11 @@
           <t>Pegah Saebi</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>pegah.saebi96@gmail.com</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>MFA Design</t>
@@ -69187,7 +69303,7 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Own site (pegahsaebi.com) found via web search but could not be resolved by this tool's fetcher (DNS failure) — try visiting manually</t>
+          <t>Email confirmed by user (site was unresolvable by this tool's fetcher)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email discovery pass for VCU: 6/13 confirmed emails
Found emails for Aya Khalife, Rebecca Oh, David Guarnizo, Tyna Ontko,
Molly Garrett, and Amy Duval. Corrected a source misspelling (Suzy
Slykin -> Suzy Lykins). Two emails were text-obfuscated on the
student's own site rather than real mailto: links; one required the
new interactive_email_finder.py tool to surface.

Added interactive_email_finder.py: a Playwright-driven fallback that
hovers/clicks contact affordances on a page before extracting emails,
for portfolio sites where a plain fetch or crawl4ai's passive render
finds nothing. Filters out site-builder placeholder addresses.
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -79333,7 +79333,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>No email found via web search — LinkedIn, Pinterest, Facebook, and ethicaljewelry.org VCU chapter page all confirmed her identity (metal/glass artist, Craft/Material Studies MFA) but none published a direct email; no personal portfolio site found</t>
         </is>
       </c>
     </row>
@@ -79368,7 +79368,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>No email found — confirmed real via VCU Scholars Compass thesis record and VCUarts Sculpture Instagram feature; aneuscheler.info found but appears to be an unrelated site with no VCU/contact content; no personal portfolio site found</t>
         </is>
       </c>
     </row>
@@ -79378,7 +79378,11 @@
           <t>Aya Khalife</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>khalifehaya7@gmail.com</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MFA Fine Arts</t>
@@ -79389,7 +79393,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.ayakhalife.com/</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>VCU</t>
@@ -79403,20 +79411,20 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page (collaborative piece, multiple credited artists); likely incomplete relative to full graduating cohort</t>
+          <t>Email confirmed by user (portfolio site ayakhalife.com, JS-rendered Readymag site, personal email surfaced via 'Reach out' mailto link only visible on hover — not captured by automated fetch/crawl4ai)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Suzy Slykin</t>
+          <t>Suzy Lykins</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting and Printmaking</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -79438,7 +79446,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page (collaborative piece, multiple credited artists); likely incomplete relative to full graduating cohort</t>
+          <t>Name corrected from 'Suzy Slykin' (source ICA caption misspelling) to 'Suzy Lykins', confirmed via matching thesis title 'Post Opera' on VCU Scholars Compass (scholarscompass.vcu.edu/etd/7995/). No email found via web search — no personal site/social found under correct spelling</t>
         </is>
       </c>
     </row>
@@ -79448,10 +79456,14 @@
           <t>Rebecca Oh</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>rebeccaohart@gmail.com</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting and Printmaking</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -79459,7 +79471,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>http://www.rebeccaoh.com/</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>VCU</t>
@@ -79473,7 +79489,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page (collaborative piece, multiple credited artists); likely incomplete relative to full graduating cohort</t>
+          <t>Email found via web search (own site rebeccaoh.com/about, verified in raw HTML: 'Feel free to e-mail the artist at rebeccaohart@gmail.com')</t>
         </is>
       </c>
     </row>
@@ -79483,10 +79499,14 @@
           <t>David Guarnizo</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>guarnizode@vcu.edu</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Photography and Film</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -79494,7 +79514,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://arts.vcu.edu/directory/david-guarnizo/</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>VCU</t>
@@ -79508,7 +79532,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>Email found via web search (VCU School of the Arts directory page, verified in raw HTML)</t>
         </is>
       </c>
     </row>
@@ -79518,10 +79542,14 @@
           <t>Tyna Ontko</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ontkotyna@gmail.com</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Sculpture and Extended Media</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -79529,7 +79557,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://tynaontko.com/</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>VCU</t>
@@ -79543,7 +79575,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>Email found via web search (own site tynaontko.com/contact, address was obfuscated as 'ontkotyna(at)gmail(dot)com' in page text, deobfuscated)</t>
         </is>
       </c>
     </row>
@@ -79556,7 +79588,7 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting and Printmaking</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -79578,7 +79610,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>No email found via web search — confirmed real (BFA 2021 UCF, painter) via ArtFields competition page and Instagram, but no personal portfolio site found and no email published anywhere</t>
         </is>
       </c>
     </row>
@@ -79591,7 +79623,7 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Craft/Material Studies</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -79613,7 +79645,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>No email found via web search — confirmed real via MutualArt profile and LinkedIn (Textile Artist and Designer), but no personal portfolio site found and no email published anywhere</t>
         </is>
       </c>
     </row>
@@ -79626,7 +79658,7 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Craft/Material Studies</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -79648,7 +79680,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>No email found via web search — confirmed real (BFA Ceramics, Indiana University Southeast 2020) via Alma's Gallery product page and Instagram (@brooklingrantzceramics), but no personal website found and no email published anywhere</t>
         </is>
       </c>
     </row>
@@ -79658,10 +79690,14 @@
           <t>Molly Garrett</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>hi@mollygarrett.com</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Graphic Design</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -79669,7 +79705,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://mollygarrett.com/</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>VCU</t>
@@ -79683,7 +79723,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>Email found via web search (own site mollygarrett.com/contact, address was obfuscated as 'hi [at] mollygarrett.com' in page text, deobfuscated)</t>
         </is>
       </c>
     </row>
@@ -79696,7 +79736,7 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Painting and Printmaking</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -79718,7 +79758,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page (collaborative piece, multiple credited artists); likely incomplete relative to full graduating cohort</t>
+          <t>No email found via web search — common name causes ambiguity (an unrelated NYC art historian also named Alex Bacon has a similar-looking alex-bacon.com site, confirmed NOT this person). Confirmed real via VCU Scholars Compass thesis 'Wiring Attachment' by Alexander Kunin Bacon and Bond Millen Gallery bio, but no personal site/email found for the correct person</t>
         </is>
       </c>
     </row>
@@ -79728,10 +79768,14 @@
           <t>Amy Duval</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>amys.duval@gmail.com</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MFA Fine Arts</t>
+          <t>MFA Craft/Material Studies</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -79739,7 +79783,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.duvalceramics.ca/</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>VCU</t>
@@ -79753,7 +79801,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Name only, from artwork photo caption credit on ICA exhibition page; likely incomplete relative to full graduating cohort</t>
+          <t>Email found via web search (own site duvalceramics.ca/contact, JS-rendered — found via interactive Playwright probe of the contact form page)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email discovery pass for Ohio State: 4/21 confirmed (2025 cohort only)
Found emails for Mandy Darrington, William Evans, Andrew Mehall, and
Ivan David Ng from the confident 2025 cohort. Left the 8 UNVERIFIED
2026 cohort names untouched after catching a near-miss: an OSU
directory hit matched only on surname (a different Estabrook, a
Lecturer) not the full reconstructed name, and was correctly not used.

Several web-search-surfaced OSU directory URLs turned out to be stale
404s -- confirms the project's "verify before trusting a URL" rule
applies to search snippets too, not just source docs.
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students.xlsx
@@ -14633,7 +14633,11 @@
           <t>Mandy Darrington</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>mandylynndarrington@gmail.com</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MFA Studio Art</t>
@@ -14646,7 +14650,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://www.mandydarrington.com/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -14662,7 +14666,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>Email found via web search (own site mandydarrington.com/about, obfuscated as 'mandylynndarrington [at] gmail [dot] com', deobfuscated)</t>
         </is>
       </c>
     </row>
@@ -14685,7 +14689,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://www.annelise-duque.com/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -14701,7 +14705,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found — own site annelise-duque.com found (CV/contact pages checked directly and via interactive Playwright probe), only Squarespace placeholder text present, no personal email published</t>
         </is>
       </c>
     </row>
@@ -14711,7 +14715,11 @@
           <t>William Evans</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>evans_william@live.com</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MFA Studio Art</t>
@@ -14724,7 +14732,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://www.williamevans.studio/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -14740,7 +14748,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>Email found via web search (own site williamevans.studio/about, plain text)</t>
         </is>
       </c>
     </row>
@@ -14779,7 +14787,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found — confirmed real (ceramic artist, Bronx NY, BFA SUNY New Paltz) via Instagram and Clay Art Center residency mentions; OSU directory profile page 404s, no personal site found</t>
         </is>
       </c>
     </row>
@@ -14802,7 +14810,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://www.josiahjamison.com/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -14818,7 +14826,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found — own site josiahjamison.com found (about/CV pages checked), only Squarespace placeholder text present, no personal email published</t>
         </is>
       </c>
     </row>
@@ -14857,7 +14865,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found via web search — no personal site surfaced; note a 'Matthew Machado' also appears as an OSU Art Department Lecturer, possibly the same person post-graduation, but not confirmed as the same identity so not used</t>
         </is>
       </c>
     </row>
@@ -14867,7 +14875,11 @@
           <t>Andrew Mehall</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>mehall.11@osu.edu</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MFA Studio Art</t>
@@ -14880,7 +14892,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://art.osu.edu/people/mehall.11</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -14896,7 +14908,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>Email found via web search (OSU Department of Art directory profile, institutional address, verified in raw HTML)</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14931,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://livablefuturesnow.org/zazanaylor</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -14935,7 +14947,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found — confirmed real (Zachary Naylor, b. 1993 Waterbury CT) via Livable Futures artist page, only Squarespace placeholder text present; OSU directory profile page 404s</t>
         </is>
       </c>
     </row>
@@ -14945,10 +14957,14 @@
           <t>Ivan David Ng</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>info@ivandavidng.com</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MFA Studio Art</t>
+          <t>MFA Drawing and Painting</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -14958,7 +14974,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://www.ivandavidng.com/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -14974,7 +14990,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>Email found via web search (own site ivandavidng.com/about, plain text)</t>
         </is>
       </c>
     </row>
@@ -14987,7 +15003,7 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MFA Studio Art</t>
+          <t>MFA Art and Technology</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -14997,7 +15013,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>http://www.julianrobbins.art/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -15013,7 +15029,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found — own site julianrobbinsart.wordpress.com/julianrobbins.art found, checked via interactive Playwright probe, no email/contact affordance found; OSU directory profile page 404s</t>
         </is>
       </c>
     </row>
@@ -15036,7 +15052,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://www.isabellasaraceni.com/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -15052,7 +15068,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found — own site isabellasaraceni.com found, checked via interactive Playwright probe, no email/contact affordance found; OSU directory profile page 404s</t>
         </is>
       </c>
     </row>
@@ -15065,7 +15081,7 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MFA Studio Art</t>
+          <t>MFA Studio Art (Ceramics)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -15075,7 +15091,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://art.osu.edu/events/mfa-thesis-exhibition-desire-lines</t>
+          <t>https://www.alextrippe.com/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -15091,7 +15107,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found — own site alextrippe.com found (full name Alexandra Trippe), checked via interactive Playwright probe, no email/contact affordance found; OSU directory profile page 404s</t>
         </is>
       </c>
     </row>
@@ -15130,7 +15146,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Name only, from 'Participating Artists' list; no email/portfolio published on source page</t>
+          <t>No email found via web search — confirmed real via First-Year MFA Show and Desire Lines exhibition mentions, but no personal site found and no email published anywhere</t>
         </is>
       </c>
     </row>

</xml_diff>